<commit_message>
4.7.2e interim 2 part testin on console only
</commit_message>
<xml_diff>
--- a/output/AIPN_Enriched.xlsx
+++ b/output/AIPN_Enriched.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,13 +43,6 @@
     <font>
       <b val="1"/>
       <color rgb="00000000"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="10"/>
-      <sz val="12"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <name val="Consolas"/>
@@ -125,11 +118,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -161,16 +153,16 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,13 +174,9 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -551,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -613,142 +601,152 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Local Knowledge - No MPN for Parts Master lookup</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Local Knowledge - Not in Parts Master</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Identity Candidates Discovered</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>8</v>
-      </c>
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Providers</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>DigiKey, Mouser, TME</t>
-        </is>
+          <t>Identity Candidates Discovered</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>DigiKey provider activity</t>
+          <t>Providers</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>13 calls; 9.0 s cumulative; 0 errors; 0 skipped</t>
+          <t>DigiKey, Mouser, TME</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Mouser provider activity</t>
+          <t>DigiKey provider activity</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>11 calls; 8.4 s cumulative; 0 errors; 0 skipped</t>
+          <t>3 calls; 1.0 s cumulative; 0 errors; 0 skipped</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TME provider activity</t>
+          <t>Mouser provider activity</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>11 calls; 14.8 s cumulative; 2 errors; 0 skipped</t>
+          <t>3 calls; 3.0 s cumulative; 0 errors; 0 skipped</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Provider operations</t>
+          <t>TME provider activity</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>3 calls; 1.4 s cumulative; 3 errors; 0 skipped</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Knowledge Base results</t>
+          <t>Provider operations</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Live API results</t>
+          <t>Knowledge Base results</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Timing note</t>
+          <t>Live API results</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Provider times are cumulative and may overlap because providers are queried concurrently.</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Review Rule</t>
+          <t>Timing note</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>DNP rows are reviewed like fitted rows; DNP remains assembly context.</t>
+          <t>Provider times are cumulative and may overlap because providers are queried concurrently.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Review Rule</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DNP rows are reviewed like fitted rows; DNP remains assembly context.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>PDC reports evidence and exceptions only; no automatic engineering approval.</t>
         </is>
@@ -770,7 +768,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
@@ -780,7 +778,7 @@
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
@@ -1187,11 +1185,7 @@
           <t>Hirose</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>BM28B0.6-6DS/2-0.35V(51)</t>
-        </is>
-      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="11" t="inlineStr">
         <is>
           <t>Review Required</t>
@@ -1209,7 +1203,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Identity requires review; No provider identity match confirmed; Provider collection incomplete</t>
+          <t>MPN missing - candidate recovered: BM28B0.6-6DS_2-0.35V_51_; 2 identity/variant candidate(s) discovered; Identity requires review; No provider identity match confirmed; Provider collection incomplete</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1231,7 +1225,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Not in Parts Master</t>
+          <t>No MPN for Parts Master lookup</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
@@ -1333,7 +1327,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>8 identity/variant candidate(s) discovered; Provider collection incomplete</t>
+          <t>Provider collection incomplete</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1545,7 +1539,7 @@
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="36" customWidth="1" min="12" max="12"/>
   </cols>
@@ -1623,15 +1617,19 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>BM28B0.6-6DS/2-0.35V(51)</t>
+          <t>BM28B0.6-6DS_2-0.35V_51_</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Identity requires review; No provider identity match confirmed; Provider collection incomplete</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>MPN missing - candidate recovered: BM28B0.6-6DS_2-0.35V_51_; 2 identity/variant candidate(s) discovered; Identity requires review; No provider identity match confirmed; Provider collection incomplete</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>BM28B0.6-6DS_2-0.35V_51_; BM28B0.6-6DS/2-0.35V(51)</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Review Required</t>
@@ -1648,7 +1646,11 @@
           <t>BoardConn_6S_BM28B0.6-6DS2-0.35V51:BoardConn_6S_BM28B0.6-6DS2-0.35V51</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Not assessed; Consistent - MPN referenced by footprint</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr"/>
     </row>
@@ -1852,7 +1854,7 @@
       <c r="R2" s="2" t="inlineStr"/>
       <c r="S2" s="2" t="inlineStr"/>
       <c r="T2" s="17" t="n">
-        <v>46264.77550925926</v>
+        <v>46264.9959837963</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
@@ -2984,7 +2986,7 @@
       <c r="R17" s="2" t="inlineStr"/>
       <c r="S17" s="2" t="inlineStr"/>
       <c r="T17" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
@@ -3048,7 +3050,7 @@
       <c r="R18" s="2" t="inlineStr"/>
       <c r="S18" s="2" t="inlineStr"/>
       <c r="T18" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
@@ -3112,7 +3114,7 @@
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr"/>
       <c r="T19" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
@@ -3176,7 +3178,7 @@
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
       <c r="T20" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
@@ -3240,7 +3242,7 @@
       <c r="R21" s="2" t="inlineStr"/>
       <c r="S21" s="2" t="inlineStr"/>
       <c r="T21" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
@@ -3304,7 +3306,7 @@
       <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -3368,7 +3370,7 @@
       <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="inlineStr"/>
       <c r="T23" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
@@ -3432,7 +3434,7 @@
       <c r="R24" s="2" t="inlineStr"/>
       <c r="S24" s="2" t="inlineStr"/>
       <c r="T24" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -3496,7 +3498,7 @@
       <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
       <c r="T25" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
@@ -3560,7 +3562,7 @@
       <c r="R26" s="2" t="inlineStr"/>
       <c r="S26" s="2" t="inlineStr"/>
       <c r="T26" s="17" t="n">
-        <v>46264.77532407407</v>
+        <v>46264.99594907407</v>
       </c>
     </row>
   </sheetData>
@@ -3574,20 +3576,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
@@ -3667,46 +3669,42 @@
     </row>
     <row r="2">
       <c r="A2" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
+          <t>Hirose</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2.2uH</t>
+          <t>BM28B0.6-6DS_2-0.35V_51_</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
+          <t>BoardConn_6S_BM28B0.6-6DS2-0.35V51:BoardConn_6S_BM28B0.6-6DS2-0.35V51</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Abracon LLC</t>
+          <t>Hirose</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>AOTA-N160808S-1R0MT</t>
+          <t>BM28B0.6-6DS_2-0.35V_51_</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Manufacturer family discovery candidate</t>
+          <t>Recovered MPN candidate</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>DigiKey</t>
+          <t>BOM Value</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -3715,11 +3713,7 @@
           <t>Not assessed</t>
         </is>
       </c>
-      <c r="L2" s="18" t="inlineStr">
-        <is>
-          <t>https://abracon.com/datasheets/AOTA-N160808S.pdf</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Review Required</t>
@@ -3727,47 +3721,43 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
+          <t>Input MPN is blank; candidate recovered from BOM context. Review required.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
+          <t>Hirose</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2.2uH</t>
+          <t>BM28B0.6-6DS_2-0.35V_51_</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
+          <t>BoardConn_6S_BM28B0.6-6DS2-0.35V51:BoardConn_6S_BM28B0.6-6DS2-0.35V51</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>ABRACON</t>
+          <t>Hirose Connector</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>AOTA-N160808S-1R0MT</t>
+          <t>BM28B0.6-6DS/2-0.35V(51)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Manufacturer family discovery candidate</t>
+          <t>Recovered MPN candidate</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -3778,14 +3768,10 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L3" s="18" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/datasheet/3/184/1/AOTA_N160808S.pdf</t>
-        </is>
-      </c>
+          <t>Consistent - MPN referenced by footprint</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Review Required</t>
@@ -3793,417 +3779,11 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2.2uH</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Abracon LLC</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-R24MT</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturer family discovery candidate</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L4" s="18" t="inlineStr">
-        <is>
-          <t>https://abracon.com/datasheets/AOTA-N160808S.pdf</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>2.2uH</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>ABRACON</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-R24MT</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturer family discovery candidate</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L5" s="18" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/datasheet/3/184/1/AOTA_N160808S.pdf</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2.2uH</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Abracon LLC</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-R47MT</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturer family discovery candidate</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L6" s="18" t="inlineStr">
-        <is>
-          <t>https://abracon.com/datasheets/AOTA-N160808S.pdf</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>2.2uH</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>ABRACON</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-R47MT</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturer family discovery candidate</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L7" s="18" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/datasheet/3/184/1/AOTA_N160808S.pdf</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>2.2uH</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Abracon LLC</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-R56MT</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturer family discovery candidate</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L8" s="18" t="inlineStr">
-        <is>
-          <t>https://abracon.com/datasheets/AOTA-N160808S.pdf</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Abracon</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-2R2MT</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2.2uH</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Inductor_SMD:L_0603_1608Metric</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>ABRACON</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>AOTA-N160808S-R56MT</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Manufacturer family discovery candidate</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Mouser</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Not assessed</t>
-        </is>
-      </c>
-      <c r="L9" s="18" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/datasheet/3/184/1/AOTA_N160808S.pdf</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Review Required</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Discovered from family key AOTAN160808 after 35% right-side reduction. Candidate requires manufacturer-document/order-table verification.</t>
+          <t>Provider supports BOM-context MPN candidate; review required.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>